<commit_message>
update memory fragment calculate / update data
</commit_message>
<xml_diff>
--- a/Data/Equipment.xlsx
+++ b/Data/Equipment.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CombatCalculatorTest\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CombatCalculatorTest\Data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F557755B-D375-48E4-9867-9EF4E75142E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49BE3F4F-3A63-4CEF-A917-87A33E7021F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17520" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="23865" windowHeight="16320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Equipment" sheetId="1" r:id="rId1"/>
@@ -21,6 +21,53 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>何巧薇</author>
+  </authors>
+  <commentList>
+    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{FC407B38-5D38-496A-8DC8-4BA3D3C37CE3}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="細明體"/>
+            <family val="3"/>
+            <charset val="136"/>
+          </rPr>
+          <t>何巧薇</t>
+        </r>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t>:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Tahoma"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">
+AttackFlat
+DefenseFlat
+HealthPointFlat</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
   <si>
@@ -73,7 +120,7 @@
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
   <si>
-    <t>ATK_FLAT</t>
+    <t>AttackFlat</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
 </sst>
@@ -81,7 +128,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="7" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -108,6 +155,27 @@
       <name val="Arial"/>
       <family val="2"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Tahoma"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="細明體"/>
+      <family val="3"/>
+      <charset val="136"/>
     </font>
   </fonts>
   <fills count="4">
@@ -362,7 +430,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
@@ -414,6 +482,8 @@
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+  <legacyDrawing r:id="rId2"/>
 </worksheet>
 </file>
 

</xml_diff>

<commit_message>
update data and schema
</commit_message>
<xml_diff>
--- a/Data/Equipment.xlsx
+++ b/Data/Equipment.xlsx
@@ -1,16 +1,10 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="7" rupBuild="9302"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\CombatCalculatorTest\Data\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{49BE3F4F-3A63-4CEF-A917-87A33E7021F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="780" yWindow="780" windowWidth="23865" windowHeight="16320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="23865" windowHeight="16320" activeTab="2"/>
   </bookViews>
   <sheets>
     <sheet name="Equipment" sheetId="1" r:id="rId1"/>
@@ -22,12 +16,12 @@
 </file>
 
 <file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
-<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <authors>
     <author>何巧薇</author>
   </authors>
   <commentList>
-    <comment ref="D1" authorId="0" shapeId="0" xr:uid="{FC407B38-5D38-496A-8DC8-4BA3D3C37CE3}">
+    <comment ref="D1" authorId="0">
       <text>
         <r>
           <rPr>
@@ -69,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="20">
   <si>
     <t>EquipmentId</t>
   </si>
@@ -78,12 +72,6 @@
   </si>
   <si>
     <t>SlotType</t>
-  </si>
-  <si>
-    <t>MainStatType</t>
-  </si>
-  <si>
-    <t>MainStatValue</t>
   </si>
   <si>
     <t>EffectIndex</t>
@@ -123,12 +111,29 @@
     <t>AttackFlat</t>
     <phoneticPr fontId="2" type="noConversion"/>
   </si>
+  <si>
+    <t>StatTypeId</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>Value</t>
+    <phoneticPr fontId="2" type="noConversion"/>
+  </si>
+  <si>
+    <t>AttackFlat</t>
+  </si>
+  <si>
+    <t>Flat</t>
+  </si>
+  <si>
+    <t>StaticBase</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -177,8 +182,13 @@
       <family val="3"/>
       <charset val="136"/>
     </font>
+    <font>
+      <sz val="10"/>
+      <color theme="1"/>
+      <name val="Arial"/>
+    </font>
   </fonts>
-  <fills count="4">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -197,8 +207,14 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD9EAD3"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -206,16 +222,41 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color rgb="FFCCCCCC"/>
+      </left>
+      <right style="medium">
+        <color rgb="FFCCCCCC"/>
+      </right>
+      <top style="medium">
+        <color rgb="FFCCCCCC"/>
+      </top>
+      <bottom style="medium">
+        <color rgb="FFCCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="一般" xfId="0" builtinId="0"/>
@@ -430,11 +471,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="16.140625" bestFit="1" customWidth="1"/>
@@ -451,21 +492,21 @@
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>3</v>
+        <v>15</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>4</v>
+        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C2" s="1">
         <v>0</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="E2" s="1">
         <v>10</v>
@@ -478,6 +519,10 @@
     <row r="4" spans="1:5" x14ac:dyDescent="0.2">
       <c r="C4" s="1"/>
       <c r="D4" s="1"/>
+    </row>
+    <row r="6" spans="1:5" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
@@ -488,7 +533,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <tabColor rgb="FF999999"/>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -501,19 +546,19 @@
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>7</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>9</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.2">
@@ -529,45 +574,58 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
   <dimension ref="A1:F4"/>
   <sheetFormatPr defaultColWidth="12.5703125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="F1" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="1"/>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    </row>
+    <row r="2" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" s="6"/>
+      <c r="C2" s="6"/>
+      <c r="D2" s="7" t="b">
+        <v>0</v>
+      </c>
+      <c r="E2" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" ht="13.5" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
+      <c r="B3" s="6"/>
+      <c r="C3" s="6"/>
+      <c r="D3" s="6"/>
+      <c r="E3" s="6"/>
+      <c r="F3" s="6"/>
+    </row>
+    <row r="4" spans="1:6" ht="12.75" x14ac:dyDescent="0.2">
       <c r="E4" s="1"/>
     </row>
   </sheetData>

</xml_diff>